<commit_message>
change files from express.js  to elctron.js
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,25 +454,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>نثار احمد</v>
+        <v xml:space="preserve">کامران </v>
       </c>
       <c r="B2" t="str">
-        <v>احمدی</v>
+        <v>شکیب</v>
       </c>
       <c r="C2" t="str">
-        <v>احمدیی</v>
+        <v>شکیب</v>
       </c>
       <c r="D2" t="str">
-        <v>سید</v>
+        <v>سید محمد</v>
       </c>
       <c r="E2" t="str">
         <v>توخی</v>
       </c>
       <c r="F2" t="str">
-        <v>249</v>
+        <v>1403</v>
       </c>
       <c r="G2" t="str">
-        <v>959</v>
+        <v>2004</v>
       </c>
       <c r="H2" t="str">
         <v>هرات</v>
@@ -481,10 +481,10 @@
         <v>هرات</v>
       </c>
       <c r="J2" t="str">
-        <v>9409</v>
+        <v>12</v>
       </c>
       <c r="K2" t="str">
-        <v>هراتت</v>
+        <v>دوشنبه 21 حمل</v>
       </c>
       <c r="L2" t="str">
         <v>دری</v>
@@ -505,9 +505,1237 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B3" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C3" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D3" t="str">
+        <v>سید محمد</v>
+      </c>
+      <c r="E3" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1404</v>
+      </c>
+      <c r="G3" t="str">
+        <v>123</v>
+      </c>
+      <c r="H3" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I3" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="J3" t="str">
+        <v>12</v>
+      </c>
+      <c r="K3" t="str">
+        <v>21 حمل ساعت 4:30</v>
+      </c>
+      <c r="L3" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M3" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N3" t="str">
+        <v>30</v>
+      </c>
+      <c r="O3" t="str">
+        <v>P2400001</v>
+      </c>
+      <c r="P3">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>کامران 2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C4" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D4" t="str">
+        <v>سید محمد</v>
+      </c>
+      <c r="E4" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1404</v>
+      </c>
+      <c r="G4" t="str">
+        <v>123</v>
+      </c>
+      <c r="H4" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I4" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="J4" t="str">
+        <v>12</v>
+      </c>
+      <c r="K4" t="str">
+        <v>21 حمل ساعت 4:30</v>
+      </c>
+      <c r="L4" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M4" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N4" t="str">
+        <v>30</v>
+      </c>
+      <c r="O4" t="str">
+        <v>P2400002</v>
+      </c>
+      <c r="P4">
+        <v>30</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v xml:space="preserve">کامران </v>
+      </c>
+      <c r="B5" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C5" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D5" t="str">
+        <v>شیبک</v>
+      </c>
+      <c r="E5" t="str">
+        <v>شیبک</v>
+      </c>
+      <c r="F5" t="str">
+        <v>009</v>
+      </c>
+      <c r="G5" t="str">
+        <v>090</v>
+      </c>
+      <c r="H5" t="str">
+        <v>هرت</v>
+      </c>
+      <c r="I5" t="str">
+        <v>هراهت</v>
+      </c>
+      <c r="J5" t="str">
+        <v>09</v>
+      </c>
+      <c r="K5" t="str">
+        <v>ه</v>
+      </c>
+      <c r="L5" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M5" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N5" t="str">
+        <v>30</v>
+      </c>
+      <c r="O5" t="str">
+        <v>P2400003</v>
+      </c>
+      <c r="P5">
+        <v>30</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v xml:space="preserve">کامران </v>
+      </c>
+      <c r="B6" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C6" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D6" t="str">
+        <v>شیبک</v>
+      </c>
+      <c r="E6" t="str">
+        <v>شیبک</v>
+      </c>
+      <c r="F6" t="str">
+        <v>009</v>
+      </c>
+      <c r="G6" t="str">
+        <v>090</v>
+      </c>
+      <c r="H6" t="str">
+        <v>هرت</v>
+      </c>
+      <c r="I6" t="str">
+        <v>هراهت</v>
+      </c>
+      <c r="J6" t="str">
+        <v>09</v>
+      </c>
+      <c r="K6" t="str">
+        <v>ه</v>
+      </c>
+      <c r="L6" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M6" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N6" t="str">
+        <v>30</v>
+      </c>
+      <c r="O6" t="str">
+        <v>P2400004</v>
+      </c>
+      <c r="P6">
+        <v>30</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B7" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C7" t="str">
+        <v>شنیسبت</v>
+      </c>
+      <c r="D7" t="str">
+        <v>نشبست</v>
+      </c>
+      <c r="E7" t="str">
+        <v>نشیستب</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0909</v>
+      </c>
+      <c r="G7" t="str">
+        <v>090</v>
+      </c>
+      <c r="H7" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I7" t="str">
+        <v>رهتنتشب</v>
+      </c>
+      <c r="J7" t="str">
+        <v>نتن</v>
+      </c>
+      <c r="K7" t="str">
+        <v>ننشیستنبت</v>
+      </c>
+      <c r="L7" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M7" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N7" t="str">
+        <v>30</v>
+      </c>
+      <c r="O7" t="str">
+        <v>P24000005</v>
+      </c>
+      <c r="P7">
+        <v>30</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>askdfj</v>
+      </c>
+      <c r="B8" t="str">
+        <v>kasdjf</v>
+      </c>
+      <c r="C8" t="str">
+        <v>aksfdj</v>
+      </c>
+      <c r="D8" t="str">
+        <v>kasdjf</v>
+      </c>
+      <c r="E8" t="str">
+        <v>kasjdf</v>
+      </c>
+      <c r="F8" t="str">
+        <v>090</v>
+      </c>
+      <c r="G8" t="str">
+        <v>0909</v>
+      </c>
+      <c r="H8" t="str">
+        <v>kajsdfk</v>
+      </c>
+      <c r="I8" t="str">
+        <v>kaksfj</v>
+      </c>
+      <c r="J8" t="str">
+        <v>kajsfd</v>
+      </c>
+      <c r="K8" t="str">
+        <v>kasjfdkj</v>
+      </c>
+      <c r="L8" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M8" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N8" t="str">
+        <v>30</v>
+      </c>
+      <c r="O8" t="str">
+        <v>P24011111</v>
+      </c>
+      <c r="P8">
+        <v>30</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>askdfj2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>222</v>
+      </c>
+      <c r="C9" t="str">
+        <v>aksfdj</v>
+      </c>
+      <c r="D9" t="str">
+        <v>kasdjf</v>
+      </c>
+      <c r="E9" t="str">
+        <v>kasjdf</v>
+      </c>
+      <c r="F9" t="str">
+        <v>090</v>
+      </c>
+      <c r="G9" t="str">
+        <v>0909</v>
+      </c>
+      <c r="H9" t="str">
+        <v>kajsdfk</v>
+      </c>
+      <c r="I9" t="str">
+        <v>kaksfj</v>
+      </c>
+      <c r="J9" t="str">
+        <v>kajsfd</v>
+      </c>
+      <c r="K9" t="str">
+        <v>kasjfdkj</v>
+      </c>
+      <c r="L9" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M9" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N9" t="str">
+        <v>30</v>
+      </c>
+      <c r="O9" t="str">
+        <v>P24011112</v>
+      </c>
+      <c r="P9">
+        <v>30</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B10" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="C10" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D10" t="str">
+        <v>سیدمحمد</v>
+      </c>
+      <c r="E10" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F10" t="str">
+        <v>1404</v>
+      </c>
+      <c r="G10" t="str">
+        <v>13983</v>
+      </c>
+      <c r="H10" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I10" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="J10" t="str">
+        <v>90924</v>
+      </c>
+      <c r="K10" t="str">
+        <v>روز دوشنبه</v>
+      </c>
+      <c r="L10" t="str">
+        <v>دری</v>
+      </c>
+      <c r="M10" t="str">
+        <v>آموزشگاه عالی امید افغانستان</v>
+      </c>
+      <c r="N10" t="str">
+        <v>30</v>
+      </c>
+      <c r="O10" t="str">
+        <v>P24011113</v>
+      </c>
+      <c r="P10">
+        <v>30</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F11" t="str">
+        <v>1404</v>
+      </c>
+      <c r="G11" t="str">
+        <v>1383</v>
+      </c>
+      <c r="H11" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I11" t="str">
+        <v>هارت</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>صبا</v>
+      </c>
+      <c r="L11" t="str">
+        <v>دری</v>
+      </c>
+      <c r="N11" t="str">
+        <v>50</v>
+      </c>
+      <c r="O11" t="str">
+        <v>P24055555</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>کامران 2</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1404</v>
+      </c>
+      <c r="G12" t="str">
+        <v>1383</v>
+      </c>
+      <c r="H12" t="str">
+        <v>هرات</v>
+      </c>
+      <c r="I12" t="str">
+        <v>هارت</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>صبا</v>
+      </c>
+      <c r="L12" t="str">
+        <v>دری</v>
+      </c>
+      <c r="N12" t="str">
+        <v>50</v>
+      </c>
+      <c r="O12" t="str">
+        <v>P24055556</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v>O00NaN</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v>O242424</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>علی</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>احمدی</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v>O242425</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v>O242426</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v>توخی</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v>O242427</v>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v>O242428</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v>O242429</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>O242430</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v>سیدم</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v>O242431</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v>سید</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v>O242432</v>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v>سی</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v>O242433</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>سی</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v>O242434</v>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>علی</v>
+      </c>
+      <c r="B25" t="str">
+        <v>سید</v>
+      </c>
+      <c r="C25" t="str">
+        <v>سیدی</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>تخ</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v>P2404043</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v>P2404044</v>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v>P2404045</v>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>کامران</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>شکیب</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v>P2404046</v>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>